<commit_message>
Update FixedRadioFluro test data templates to reflect changes in measurement parameters, including adjustments to FFD values, observed shifts, and edge shifts. Standardize tolerance values and improve clarity in measurement dimensions. Introduce new script for generating templates with consistent formatting and structure.
</commit_message>
<xml_diff>
--- a/public/templates/Radiography_Mobile_Template.xlsx
+++ b/public/templates/Radiography_Mobile_Template.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Test Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Sample" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -432,6 +433,9 @@
       <c r="I2" t="str">
         <v>TF Required</v>
       </c>
+      <c r="J2" t="str">
+        <v>TF At kVp</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -461,6 +465,9 @@
       <c r="I3" t="str">
         <v>2.5</v>
       </c>
+      <c r="J3" t="str">
+        <v>80</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -527,7 +534,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>FCD</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B8" t="str">
         <v>kV</v>
@@ -624,7 +631,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>FFD</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B14" t="str">
         <v>Tol Operator</v>
@@ -725,7 +732,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>FCD</v>
+        <v>FFD (cm)</v>
       </c>
       <c r="B19" t="str">
         <v>kV</v>
@@ -764,7 +771,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>FCD</v>
+        <v>FFD (cm)</v>
       </c>
       <c r="B23" t="str">
         <v>kV</v>
@@ -847,22 +854,16 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>FCD</v>
+        <v>FFD (cm)</v>
       </c>
       <c r="B28" t="str">
         <v>Focus Type</v>
       </c>
       <c r="C28" t="str">
-        <v>Stated Width</v>
+        <v>Stated Focal Spot of Tube (f)</v>
       </c>
       <c r="D28" t="str">
-        <v>Stated Height</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Measured Width</v>
-      </c>
-      <c r="F28" t="str">
-        <v>Measured Height</v>
+        <v>Measured Focal Spot (Nominal)</v>
       </c>
     </row>
     <row r="29">
@@ -878,12 +879,6 @@
       <c r="D29" t="str">
         <v/>
       </c>
-      <c r="E29" t="str">
-        <v/>
-      </c>
-      <c r="F29" t="str">
-        <v/>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -896,12 +891,6 @@
         <v/>
       </c>
       <c r="D30" t="str">
-        <v/>
-      </c>
-      <c r="E30" t="str">
-        <v/>
-      </c>
-      <c r="F30" t="str">
         <v/>
       </c>
     </row>
@@ -912,7 +901,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>FCD</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B33" t="str">
         <v>kV</v>
@@ -1033,7 +1022,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>FCD</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B39" t="str">
         <v>kV</v>
@@ -1142,7 +1131,870 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>FCD</v>
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B45" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C45" t="str">
+        <v>mA</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Time</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Workload</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Tol Value</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Tol Operator</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Location</v>
+      </c>
+      <c r="I45" t="str">
+        <v>Left</v>
+      </c>
+      <c r="J45" t="str">
+        <v>Right</v>
+      </c>
+      <c r="K45" t="str">
+        <v>Front</v>
+      </c>
+      <c r="L45" t="str">
+        <v>Back</v>
+      </c>
+      <c r="M45" t="str">
+        <v>Top</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>100</v>
+      </c>
+      <c r="B46" t="str">
+        <v>80</v>
+      </c>
+      <c r="C46" t="str">
+        <v>100</v>
+      </c>
+      <c r="D46" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="E46" t="str">
+        <v>5000</v>
+      </c>
+      <c r="F46" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="G46" t="str">
+        <v>less than or equal to</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Tube</v>
+      </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+      <c r="K46" t="str">
+        <v/>
+      </c>
+      <c r="L46" t="str">
+        <v/>
+      </c>
+      <c r="M46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v/>
+      </c>
+      <c r="B47" t="str">
+        <v/>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v>Collimator</v>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+      <c r="K47" t="str">
+        <v/>
+      </c>
+      <c r="L47" t="str">
+        <v/>
+      </c>
+      <c r="M47" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M47"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M47"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TEST: ACCURACY OF OPERATING POTENTIAL</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mA Station</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Applied kV</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Tolerance Sign</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Tolerance Value</v>
+      </c>
+      <c r="H2" t="str">
+        <v>TF Measured</v>
+      </c>
+      <c r="I2" t="str">
+        <v>TF Required</v>
+      </c>
+      <c r="J2" t="str">
+        <v>TF At kVp</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>50 mA</v>
+      </c>
+      <c r="B3" t="str">
+        <v>60</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>±</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2.0</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="J3" t="str">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>100 mA</v>
+      </c>
+      <c r="B4" t="str">
+        <v>80</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>200 mA</v>
+      </c>
+      <c r="B5" t="str">
+        <v>100</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TEST: ACCURACY OF IRRADIATION TIME</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B8" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C8" t="str">
+        <v>mA</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Set Time (ms)</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Measured Time (ms)</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Tolerance Value</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>100</v>
+      </c>
+      <c r="B9" t="str">
+        <v>80</v>
+      </c>
+      <c r="C9" t="str">
+        <v>100</v>
+      </c>
+      <c r="D9" t="str">
+        <v>100</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="G9" t="str">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v>200</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>400</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TEST: OUTPUT CONSISTENCY</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Tol Operator</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Tol Value</v>
+      </c>
+      <c r="D14" t="str">
+        <v>kV</v>
+      </c>
+      <c r="E14" t="str">
+        <v>mAs</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Meas 4</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Meas 5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>100</v>
+      </c>
+      <c r="B15" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="C15" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="D15" t="str">
+        <v>80</v>
+      </c>
+      <c r="E15" t="str">
+        <v>10</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v>100</v>
+      </c>
+      <c r="E16" t="str">
+        <v>20</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TEST: CENTRAL BEAM ALIGNMENT</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>FFD (cm)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C19" t="str">
+        <v>mAs</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Observed Tilt</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Tolerance</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>100</v>
+      </c>
+      <c r="B20" t="str">
+        <v>80</v>
+      </c>
+      <c r="C20" t="str">
+        <v>10</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TEST: CONGRUENCE OF RADIATION</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>FFD (cm)</v>
+      </c>
+      <c r="B23" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C23" t="str">
+        <v>mAs</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Dimension</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Observed Shift</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Edge Shift</v>
+      </c>
+      <c r="G23" t="str">
+        <v>% FED</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Tolerance</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>100</v>
+      </c>
+      <c r="B24" t="str">
+        <v>80</v>
+      </c>
+      <c r="C24" t="str">
+        <v>10</v>
+      </c>
+      <c r="D24" t="str">
+        <v>X</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25" t="str">
+        <v>Y</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TEST: EFFECTIVE FOCAL SPOT</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>FFD (cm)</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Focus Type</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Stated Focal Spot of Tube (f)</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Measured Focal Spot (Nominal)</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>100</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Small</v>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v/>
+      </c>
+      <c r="B30" t="str">
+        <v>Large</v>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TEST: LINEARITY OF MA LOADING</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B33" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Time (sec)</v>
+      </c>
+      <c r="D33" t="str">
+        <v>mA Applied</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Tolerance</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>100</v>
+      </c>
+      <c r="B34" t="str">
+        <v>80</v>
+      </c>
+      <c r="C34" t="str">
+        <v>1</v>
+      </c>
+      <c r="D34" t="str">
+        <v>50</v>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="I34" t="str">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v>100</v>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v/>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v>200</v>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TEST: LINEARITY OF MAS LOADING STATIONS</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B39" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C39" t="str">
+        <v>mAs Applied</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Tolerance</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>100</v>
+      </c>
+      <c r="B40" t="str">
+        <v>80</v>
+      </c>
+      <c r="C40" t="str">
+        <v>10</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="H40" t="str">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v/>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v>20</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v/>
+      </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42" t="str">
+        <v>50</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TEST: RADIATION LEAKAGE LEVEL</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>FDD (cm)</v>
       </c>
       <c r="B45" t="str">
         <v>kV</v>

</xml_diff>